<commit_message>
WIP: rebase fixes, built-in visit counters, day-30 finale, scenes marked full screen
</commit_message>
<xml_diff>
--- a/content/cutie-scripts.xlsx
+++ b/content/cutie-scripts.xlsx
@@ -3862,7 +3862,7 @@
       </c>
       <c r="B25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">How many times they've talked at that time of day</t>
+          <t xml:space="preserve">How many days you've been here at that time of day</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">11-30</t>
+          <t xml:space="preserve">Day 30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
@@ -6877,11 +6877,6 @@
 {glad} [PLACEHOLDER welcome back C]</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Draft lines; replace with your own. Plays when the story is reopened on the same day.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
@@ -6914,11 +6909,6 @@
       <c r="D9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">daily, priority -1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Low priority, so a day-specific greeting wins when there is one.</t>
         </is>
       </c>
     </row>
@@ -6943,7 +6933,7 @@
   <sheetPr>
     <tabColor rgb="FFB08AD8"/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I166"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -7007,7 +6997,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Game night</t>
+          <t xml:space="preserve">game_night</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
@@ -7015,110 +7005,95 @@
           <t xml:space="preserve">Whole goal 25%</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Wow, you're already a quarter through. Good work. That's a substantial start, I'd say. Keep it up and you'll be done in no time. Shall we celebrate?</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">From the "Event cutscenes" tab</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wow, you're already a quarter through. Good work. That's a substantial start, I'd say. Keep it up and you'll be done in no time. Shall we celebrate?</t>
+          <t xml:space="preserve">Sure! But... um... how?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="D4" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure! But... um... how?</t>
+          <t xml:space="preserve">Hm... excellent question. How about we start by taking a break?</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hm... excellent question. How about we start by taking a break?</t>
+          <t xml:space="preserve">Sounds good to me.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="D6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sounds good to me.</t>
+          <t xml:space="preserve">Ryder turns on a game console and sits cross-legged in front of the couch. With a tilt of the analog stick, he sorts through a surprisingly large library of games...</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="D7" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder turns on a game console and sits cross-legged in front of the couch. With a tilt of the analog stick, he sorts through a surprisingly large library of games...</t>
+          <t xml:space="preserve">I have got to work on this backlog.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I have got to work on this backlog.</t>
+          <t xml:space="preserve">... he observes apologetically, sheepishly scratching his head before jolting to a stop on one.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="D9" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">... he observes apologetically, sheepishly scratching his head before jolting to a stop on one.</t>
+          <t xml:space="preserve">Have you ever played a fighting game before?</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Have you ever played a fighting game before?</t>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A: No</t>
         </is>
       </c>
     </row>
@@ -7130,7 +7105,7 @@
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A: No</t>
+          <t xml:space="preserve">B: Yes, and I'm good at them</t>
         </is>
       </c>
     </row>
@@ -7142,31 +7117,31 @@
       </c>
       <c r="G12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B: Yes, and I'm good at them</t>
+          <t xml:space="preserve">C: Yes, but I'm not good at them</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="D13" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
+      <c r="F13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ah, don't worry. This one is known for being beginner-friendly.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">C: Yes, but I'm not good at them</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ah, don't worry. This one is known for being beginner-friendly.</t>
+          <t xml:space="preserve">Alright, I'll try it.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="2">
@@ -7176,11 +7151,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="D15" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Oh, is that so? Then are you up for a challenge?</t>
@@ -7195,34 +7165,29 @@
     <row r="16">
       <c r="D16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Sure.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="F17" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Ah, don't worry. I can teach you... if you'd like that, I mean.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr" s="2">
+      <c r="G17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Alright, I'll try it.</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
@@ -7234,99 +7199,84 @@
       </c>
       <c r="F18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure.</t>
+          <t xml:space="preserve">Sounds good to me.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="D19" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sounds good to me.</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Then let's get started. I'll be him...</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="D20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Then let's get started. I'll be him...</t>
+          <t xml:space="preserve">Ryder selects a scholarly-looking mage with a stoic expression.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="D21" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder selects a scholarly-looking mage with a stoic expression.</t>
+          <t xml:space="preserve">Who do you want to play?</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="D22" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Who do you want to play?</t>
+          <t xml:space="preserve">Naples is an easy player for beginners to get a handle of. Would you like to try him?</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="D23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Zero December is good at ranged attacks, Lysandra is best for melee--</t>
+          <t xml:space="preserve">Sure.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="D24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I'll go with Castien.</t>
+          <t xml:space="preserve">Slowly, I get used to the game.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
@@ -7338,29 +7288,24 @@
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I pick up the nuances of the game quickly. Ryder turns out to be better than most people. Far better than I expected. What's more, he's also unexpectedly competitive. We each take turns playfully trash-talking one another. As he nearly knocks my character out, offhandedly, he remarks,</t>
+          <t xml:space="preserve">Ryder is kind, helpful, and gentle, going easy on me at first as he explains the very basics of movement, attacks, and strategy, but gradually taking off the kid gloves as I get used to the game.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="D26" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I seem to recall someone saying they were good at fighting games?</t>
+          <t xml:space="preserve">Wow, you've gotten so good already. I'm impressed.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
@@ -7372,41 +7317,31 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mind your own business.</t>
+          <t xml:space="preserve">Really? Thank you.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="D28" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I don't know. I asked if you were up for a challenge and I'm actually beginning to feel quite cruel for it.</t>
+          <t xml:space="preserve">Alright, one last thing to show you.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="D29" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">His special is almost completely powered up. I prepare to dodge the huge ball of energy as he activates it and...</t>
+          <t xml:space="preserve">Zero December is good at ranged attacks, Lysandra is best for melee--</t>
         </is>
       </c>
       <c r="G29" t="inlineStr" s="2">
@@ -7418,12 +7353,12 @@
     <row r="30">
       <c r="D30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">it flies harmlessly up into the sky?</t>
+          <t xml:space="preserve">I'll go with Castien.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="2">
@@ -7435,12 +7370,12 @@
     <row r="31">
       <c r="D31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Did you just... waste your special?</t>
+          <t xml:space="preserve">I pick up the nuances of the game quickly. Ryder turns out to be better than most people. Far better than I expected. What's more, he's also unexpectedly competitive.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
@@ -7452,12 +7387,12 @@
     <row r="32">
       <c r="D32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I... that was on purpose. I was just testing you.</t>
+          <t xml:space="preserve">We each take turns playfully trash-talking one another. As he nearly knocks my character out, offhandedly, he remarks,</t>
         </is>
       </c>
       <c r="G32" t="inlineStr" s="2">
@@ -7467,14 +7402,9 @@
       </c>
     </row>
     <row r="33">
-      <c r="D33" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Liar. So you were all talk!</t>
+          <t xml:space="preserve">I seem to recall someone saying they were good at fighting games?</t>
         </is>
       </c>
       <c r="G33" t="inlineStr" s="2">
@@ -7486,12 +7416,12 @@
     <row r="34">
       <c r="D34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">And as I say that, I swoop in while he's vulnerable and finish him off.</t>
+          <t xml:space="preserve">Mind your own business.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr" s="2">
@@ -7501,36 +7431,31 @@
       </c>
     </row>
     <row r="35">
-      <c r="D35" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Naples is an easy player for beginners to get a handle of. Would you like to try him?</t>
+          <t xml:space="preserve">I don't know. I asked if you were up for a challenge and I'm actually beginning to feel quite cruel for it.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="D36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure.</t>
+          <t xml:space="preserve">His special is almost completely powered up. I prepare to dodge the huge ball of energy as he activates it and...</t>
         </is>
       </c>
       <c r="G36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -7542,63 +7467,58 @@
       </c>
       <c r="F37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Slowly, I get used to the game. Ryder is kind, helpful, and gentle, going easy on me at first as he explains the very basics of movement, attacks, and strategy, but gradually taking off the kid gloves as I get used to the game.</t>
+          <t xml:space="preserve">it flies harmlessly up into the sky?</t>
         </is>
       </c>
       <c r="G37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="D38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wow, you've gotten so good already. I'm impressed.</t>
+          <t xml:space="preserve">Did you just... waste your special?</t>
         </is>
       </c>
       <c r="G38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="D39" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Really? Thank you.</t>
+          <t xml:space="preserve">I... that was on purpose. I was just testing you.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="D40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Alright, one last thing to show you.</t>
+          <t xml:space="preserve">Liar. So you were all talk!</t>
         </is>
       </c>
       <c r="G40" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A, C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -7610,42 +7530,47 @@
       </c>
       <c r="F41" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">And as I say that, I swoop in while he's vulnerable and finish him off.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">[PLACEHOLDER rest of the game-night scene, after "one last thing to show you"]</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Movie night</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Whole goal 50%</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr" s="2">
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">the_couch</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Whole goal 100%</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">You did it. You're more determined than I imagined, honestly. Say... are you going to let me read it now?</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">From the "Event cutscenes" tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="D44" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">I wasn't sure you could do it, but here we are. Halfway through. You're incredible. ...don't let it go to your head. Now maybe we should take a break. Would you like to watch a movie?</t>
         </is>
       </c>
     </row>
@@ -7655,81 +7580,71 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Sure!</t>
+      <c r="G45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A: Absolutely not</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="D46" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">As I leap towards the couch, Ryder grabs my arm and pulls me back, mid-air.</t>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B: Sure</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="D47" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F47" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Huh?</t>
+          <t xml:space="preserve">It was worth asking. But seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="D48" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F48" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">We... uh, need popcorn.</t>
+          <t xml:space="preserve">Glad to hear. Seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="D49" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F49" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">... Right.</t>
+          <t xml:space="preserve">I'm running out of ways to celebrate. Well, except one.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="D50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F50" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wait there.</t>
+          <t xml:space="preserve">What is it?</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="D51" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F51" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I wait approximately five minutes as Ryder finds and prepares popcorn for us. Finally he returns.</t>
+          <t xml:space="preserve">Let's sit down first...</t>
         </is>
       </c>
     </row>
@@ -7741,79 +7656,59 @@
       </c>
       <c r="F52" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Can I sit now--</t>
+          <t xml:space="preserve">On the floor again, right?</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="D53" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No! I mean. Wouldn't it be more fun to sit on the ground?</t>
+          <t xml:space="preserve">... No, on the couch.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="D54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He demonstrates by sitting cross-legged on the ground and patting the space next to him. Confused, I sit down.</t>
+          <t xml:space="preserve">Really?!</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="D55" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F55" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Okay then.</t>
+          <t xml:space="preserve">Yes, is that strange...?</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="D56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Anyway. What type of movie would you like to watch?</t>
+          <t xml:space="preserve">Considering how weird you've been about it, yeah.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="D57" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A: Romance</t>
+      <c r="F57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ah, so you noticed my aversion to sitting on it... I suppose I wanted to keep it clean since it was the first thing I ever bought for myself...</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="D58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B: Action</t>
+      <c r="F58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">But, well, there's something more important than that now.</t>
         </is>
       </c>
     </row>
@@ -7823,26 +7718,16 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C: Horror</t>
+      <c r="F59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Such as?</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="D60" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Oh? If that's the case, then... well, there's one I've been meaning to watch...</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">Well, about that... there's something I've been wanting to tell you, but I was worried about how you'd react...</t>
         </is>
       </c>
     </row>
@@ -7854,63 +7739,28 @@
       </c>
       <c r="F61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">What's it called?</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">Go on.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="D62" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The Notepad?</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I just... I think I may have fallen for you.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="D63" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Oh, that's a classic.</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I feel so safe with you. And I want you to feel like that with me. I know I can be awkward, and talk too much, but... {player}, I love you. I want you to be mine, and I want to be yours. But...</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="D64" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">That's what I heard. So shall we?</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I understand if you don't feel the same way--</t>
         </is>
       </c>
     </row>
@@ -7922,97 +7772,52 @@
       </c>
       <c r="F65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I nod and he starts the movie. He and I both intently watch a story about star-crossed lovers. As the credits roll, I'm sniffling. I look around and can't find Ryder. But then there he is with a box of tissues, also looking teary eyed.</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I close the distance between me and him and gently kiss him. His lips are soft and his body warm against mine.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="D66" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Are you okay?</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I wasn't expecting that. Do you...</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="D67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I will be. Would you like a tissue?</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I do.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="D68" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure.</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">What?</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="D69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not the best movie we could've picked for a celebration but it certainly was an experience, wasn't it?</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">I love you, too.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="D70" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I wonder if they have that movie I kept hearing about... They do!</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">I...wasn't expecting that. Why?</t>
         </is>
       </c>
     </row>
@@ -8024,29 +7829,19 @@
       </c>
       <c r="F71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Superguy?</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">The same reason you love me, dummy. You feel like home.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes, it sounds fun, doesn't it? And the ratings are very good.</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">I take his hands into mine.</t>
         </is>
       </c>
     </row>
@@ -8058,29 +7853,14 @@
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure, let's watch it then.</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">I want to be with you, too, Ryder. I'm just wondering.. what happened to the kuudere act you had at the beginning of the month?</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="D74" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">As we watch the movie, sitting on the uncomfortable hardwood floor, Ryder's eyebrows contort further and further. Afterwards, he has a solid frown on his face.</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">Huh?</t>
         </is>
       </c>
     </row>
@@ -8092,131 +7872,85 @@
       </c>
       <c r="F75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You look like you have a lot of thoughts about the movie.</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">Every few days you do this thing where you act like you're too cool for school.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="D76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I do.</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">"I suppose I can do my best to support you, but no promises made." "You're incredible. ...don't let it go to your head." And so on.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="D77" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">What a cryptic response.</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">Well... being an unabashed cheerleader isn't very cool, is it...?</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Such as...?</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="D79" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">He's supposed to be a superhero but he's causing so much trouble! Just think about all the collateral damage he left! Even assuming nobody got hurt from when he threw the villain into that skyscraper, what about taxpayer money?!</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">[PLACEHOLDER rest of the confession scene]</t>
+        </is>
+      </c>
+    </row>
+    <row r="79"/>
     <row r="80">
-      <c r="D80" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
+      <c r="A80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">movie_night</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Whole goal 50%</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">It's a movie. An explosive movie, but a movie.</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">I wasn't sure you could do it, but here we are. Halfway through. You're incredible. ...don't let it go to your head. Now maybe we should take a break. Would you like to watch a movie?</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">once</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="D81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fair enough. We won't always like the same things, I suppose.</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">Sure!</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="D82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure. I have no problem with that. None at all.</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">As I leap towards the couch, Ryder grabs my arm and pulls me back, mid-air.</t>
         </is>
       </c>
     </row>
@@ -8228,277 +7962,218 @@
       </c>
       <c r="F83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Then let's watch The Circle!</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Huh?</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="D84" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Right.</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">We... uh, need popcorn.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="D85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He says that but almost immediately as the movie starts...</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">... Right.</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="D86" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I think I should go make some popcorn.</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Wait there.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nuh-uh, you're not getting out of this one.</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">I wait approximately five minutes as Ryder finds and prepares popcorn for us. Finally he returns.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">But I--</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Can I sit now--</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="D89" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sit.</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">No! I mean. Wouldn't it be more fun to sit on the ground?</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="D90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I see...</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">He demonstrates by sitting cross-legged on the ground and patting the space next to him. Confused, I sit down.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="D91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Even so, he averts his eyes the whole movie, tensing with every jumpscare... and looking terrified out of his mind. After the movie, he's skittish.  As he's reaching in the fridge for a bottle of water, I start talking and he jumps.</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Okay then.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="D92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder? You okay?</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">Anyway. What type of movie would you like to watch?</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="D93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes, I think I'll be okay. Let's just... I think I'm going to leave the light on tonight.</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="G93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">C</t>
-        </is>
-      </c>
-    </row>
-    <row r="94"/>
+          <t xml:space="preserve">A: Romance</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B: Action</t>
+        </is>
+      </c>
+    </row>
     <row r="95">
-      <c r="A95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Froyo date</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Whole goal 75%</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">once</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">From the "Event cutscenes" tab</t>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C: Horror</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="D96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You've got three quarters of your work done. That's the vast majority! I'm honestly impressed by your dedication.</t>
+          <t xml:space="preserve">Oh? If that's the case, then... well, there's one I've been meaning to watch...</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="D97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I think that deserves a treat. How about we go for frozen yogurt?</t>
+          <t xml:space="preserve">What's it called?</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="D98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sure!</t>
+          <t xml:space="preserve">The Notepad?</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">When we arrive at the froyo place, Ryder holds the door open for me. We get tiny sample cups and push down the levers to dispense the froyo. There are twelve different flavors and we spend time diligently sampling each and every one, trying to decide which one to put in our bowl. In the end, I decide on a flavor... Then I see Ryder looking seriously pained, like he can't bear to part with any one flavor.</t>
+          <t xml:space="preserve">Oh, that's a classic.</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="D100" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Are you alright?</t>
+          <t xml:space="preserve">That's what I heard. So shall we?</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I'm fine. I'll just...</t>
+          <t xml:space="preserve">I nod and he starts the movie. He and I both intently watch a story about star-crossed lovers. As the credits roll, I'm sniffling. I look around and can't find Ryder.</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
@@ -8510,67 +8185,82 @@
       </c>
       <c r="F102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He suddenly pulls a lever, releasing salted caramel froyo into his bowl.</t>
+          <t xml:space="preserve">But then there he is with a box of tissues, also looking teary eyed.</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="D103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Wait!</t>
+          <t xml:space="preserve">Are you okay?</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="D104" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He stops and adds cake batter flavor. And then cookies and cream. He sighs with relief.</t>
+          <t xml:space="preserve">I will be. Would you like a tissue?</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">That should be fine.</t>
+          <t xml:space="preserve">Sure.</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="D106" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">When we're adding toppings, it's clear he's been struck by a similar indecision. In the end, he piles on chocolate chips, corn flakes, caramel, marshmallow sauce, and cookie dough pieces, each neatly placed in their own section of the bowl.</t>
+          <t xml:space="preserve">Not the best movie we could've picked for a celebration but it certainly was an experience, wasn't it?</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="D107" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder pays for both of us.</t>
+          <t xml:space="preserve">I wonder if they have that movie I kept hearing about... They do!</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -8582,19 +8272,24 @@
       </c>
       <c r="F108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Do you wanna go back home? We can sit on the couch, watch TV--</t>
+          <t xml:space="preserve">Superguy?</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="D109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A-ah, I think I'd prefer to eat here. Outside.</t>
+          <t xml:space="preserve">Yes, it sounds fun, doesn't it? And the ratings are very good.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8301,12 @@
       </c>
       <c r="F110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No problem.</t>
+          <t xml:space="preserve">Sure, let's watch it then.</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -8618,79 +8318,99 @@
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Is it just me or did he get weird when I mentioned the couch?</t>
+          <t xml:space="preserve">As we watch the movie, sitting on the uncomfortable hardwood floor, Ryder's eyebrows contort further and further. Afterwards, he has a solid frown on his face.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">We go outside and sit down. I dug into my frozen treat, only to eventually notice Ryder staring.</t>
+          <t xml:space="preserve">You look like you have a lot of thoughts about the movie.</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="D113" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Is there something on my face?</t>
+          <t xml:space="preserve">I do.</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes. It's right there.</t>
+          <t xml:space="preserve">What a cryptic response.</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He points at my face.</t>
+          <t xml:space="preserve">Such as...?</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="D116" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Right here?</t>
+          <t xml:space="preserve">He's supposed to be a superhero but he's causing so much trouble! Just think about all the collateral damage he left!</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="D117" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">No, there.</t>
+          <t xml:space="preserve">Even assuming nobody got hurt from when he threw the villain into that skyscraper, what about taxpayer money?!</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
@@ -8702,352 +8422,362 @@
       </c>
       <c r="F118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Here?</t>
+          <t xml:space="preserve">It's a movie. An explosive movie, but a movie.</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="D119" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ah, no, it's here...</t>
+          <t xml:space="preserve">Fair enough. We won't always like the same things, I suppose.</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="D120" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
       <c r="F120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">He reaches across the table and brushes his thumb gently near my mouth.</t>
+          <t xml:space="preserve">Sure. I have no problem with that. None at all.</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">For some reason, I can feel my face heat up.</t>
+          <t xml:space="preserve">Then let's watch The Circle!</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="D122" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sorry, I shouldn't have done that.</t>
+          <t xml:space="preserve">Right.</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="D123" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">He says that but almost immediately as the movie starts...</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="F124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">I think I should go make some popcorn.</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="D125" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">No, it's fine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="D124" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Narrator</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">But the whole time, I can't forget the way it felt when he touched me.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125"/>
+      <c r="F125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Nuh-uh, you're not getting out of this one.</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
     <row r="126">
-      <c r="A126" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">The couch</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Whole goal 100%</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">once</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">From the "Event cutscenes" tab</t>
+      <c r="F126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">But I--</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You did it. You're more determined than I imagined, honestly. Say... are you going to let me read it now?</t>
+          <t xml:space="preserve">Sit.</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="D128" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
+      <c r="F128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">I see...</t>
         </is>
       </c>
       <c r="G128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A: Absolutely not</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="D129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Even so, he averts his eyes the whole movie, tensing with every jumpscare... and looking terrified out of his mind. After the movie, he's skittish.</t>
         </is>
       </c>
       <c r="G129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B: Sure</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="D130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">It was worth asking. But seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
+          <t xml:space="preserve">As he's reaching in the fridge for a bottle of water, I start talking and he jumps.</t>
         </is>
       </c>
       <c r="G130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="D131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Glad to hear. Seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
+          <t xml:space="preserve">Ryder? You okay?</t>
         </is>
       </c>
       <c r="G131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="D132" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I'm running out of ways to celebrate. Well, except one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="D133" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">What is it?</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">Yes, I think I'll be okay. Let's just... I think I'm going to leave the light on tonight.</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
+    <row r="133"/>
     <row r="134">
-      <c r="D134" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
+      <c r="A134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">froyo_date</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Whole goal 75%</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Let's sit down first...</t>
+          <t xml:space="preserve">You've got three quarters of your work done. That's the vast majority! I'm honestly impressed by your dedication.</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">once</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="D135" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">On the floor again, right?</t>
+          <t xml:space="preserve">I think that deserves a treat. How about we go for frozen yogurt?</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">... No, on the couch.</t>
+          <t xml:space="preserve">Sure!</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Really?!</t>
+          <t xml:space="preserve">When we arrive at the froyo place, Ryder holds the door open for me. We get tiny sample cups and push down the levers to dispense the froyo.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes, is that strange...?</t>
+          <t xml:space="preserve">There are twelve different flavors and we spend time diligently sampling each and every one, trying to decide which one to put in our bowl. In the end, I decide on a flavor...</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="D139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Considering how weird you've been about it, yeah.</t>
+          <t xml:space="preserve">Then I see Ryder looking seriously pained, like he can't bear to part with any one flavor.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="D140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ah, so you noticed my aversion to sitting on it... I suppose I wanted to keep it clean since it was the first thing I ever bought for myself...</t>
+          <t xml:space="preserve">Are you alright?</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="D141" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">But, well, there's something more important than that now.</t>
+          <t xml:space="preserve">I'm fine. I'll just...</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="D142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Such as?</t>
+          <t xml:space="preserve">He suddenly pulls a lever, releasing salted caramel froyo into his bowl.</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="D143" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Well, about that... there's something I've been wanting to tell you, but I was worried about how you'd react...</t>
+          <t xml:space="preserve">Wait!</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="D144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Go on.</t>
+          <t xml:space="preserve">He stops and adds cake batter flavor. And then cookies and cream. He sighs with relief.</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="D145" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I just... I think I may have fallen for you.</t>
+          <t xml:space="preserve">That should be fine.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="D146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I feel so safe with you. And I want you to feel like that with me. I know I can be awkward, and talk too much, but... [PLAYER_NAME], I love you. I want you to be mine, and I want to be yours. But... I understand if you don't feel the same way--</t>
+          <t xml:space="preserve">When we're adding toppings, it's clear he's been struck by a similar indecision.</t>
         </is>
       </c>
     </row>
@@ -9059,19 +8789,19 @@
       </c>
       <c r="F147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I close the distance between me and him and gently kiss him. His lips are soft and his body warm against mine.</t>
+          <t xml:space="preserve">In the end, he piles on chocolate chips, corn flakes, caramel, marshmallow sauce, and cookie dough pieces, each neatly placed in their own section of the bowl.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="D148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I wasn't expecting that. Do you...</t>
+          <t xml:space="preserve">Ryder pays for both of us.</t>
         </is>
       </c>
     </row>
@@ -9083,19 +8813,14 @@
       </c>
       <c r="F149" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I do.</t>
+          <t xml:space="preserve">Do you wanna go back home? We can sit on the couch, watch TV--</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="D150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F150" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">What?</t>
+          <t xml:space="preserve">A-ah, I think I'd prefer to eat here. Outside.</t>
         </is>
       </c>
     </row>
@@ -9107,67 +8832,62 @@
       </c>
       <c r="F151" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I love you, too.</t>
+          <t xml:space="preserve">No problem.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="D152" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F152" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I...wasn't expecting that. Why?</t>
+          <t xml:space="preserve">Is it just me or did he get weird when I mentioned the couch?</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="D153" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">You</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F153" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The same reason you love me, dummy. You feel like home.</t>
+          <t xml:space="preserve">We go outside and sit down. I dug into my frozen treat, only to eventually notice Ryder staring.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="D154" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Narrator</t>
+          <t xml:space="preserve">You</t>
         </is>
       </c>
       <c r="F154" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I take his hands into mine.</t>
+          <t xml:space="preserve">Is there something on my face?</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="D155" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">You</t>
-        </is>
-      </c>
       <c r="F155" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">I want to be with you, too, Ryder. I'm just wondering.. what happened to the kuudere act you had at the beginning of the month?</t>
+          <t xml:space="preserve">Yes. It's right there.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="D156" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Ryder</t>
+          <t xml:space="preserve">Narrator</t>
         </is>
       </c>
       <c r="F156" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Huh?</t>
+          <t xml:space="preserve">He points at my face.</t>
         </is>
       </c>
     </row>
@@ -9179,34 +8899,92 @@
       </c>
       <c r="F157" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Every few days you do this thing where you act like you're too cool for school. "I suppose I can do my best to support you, but no promises made." "You're incredible. ...don't let it go to your head." And so on.</t>
+          <t xml:space="preserve">Right here?</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="D158" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Ryder</t>
-        </is>
-      </c>
       <c r="F158" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Well... being an unabashed cheerleader isn't very cool, is it...?</t>
+          <t xml:space="preserve">No, there.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="D159" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Here?</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="F160" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Ah, no, it's here...</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="D161" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">[PLACEHOLDER rest of the confession scene]</t>
-        </is>
-      </c>
-    </row>
+      <c r="F161" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">He reaches across the table and brushes his thumb gently near my mouth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="D162" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">For some reason, I can feel my face heat up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="F163" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sorry, I shouldn't have done that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="D164" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No, it's fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="D165" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">But the whole time, I can't forget the way it felt when he touched me.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166"/>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="D2:D500">

</xml_diff>

<commit_message>
Workbook: Picture column in Scenes
</commit_message>
<xml_diff>
--- a/content/cutie-scripts.xlsx
+++ b/content/cutie-scripts.xlsx
@@ -3379,7 +3379,7 @@
   <sheetPr>
     <tabColor rgb="FFC9C2D4"/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3387,10 +3387,11 @@
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="80" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="80" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3421,20 +3422,25 @@
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Picture</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Line</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Choice</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Options</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -3461,12 +3467,12 @@
           <t xml:space="preserve">smile</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Halfway! Want to watch a movie?</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr" s="2">
+      <c r="I2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
         </is>
@@ -3478,7 +3484,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr" s="2">
+      <c r="H3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A: Romance</t>
         </is>
@@ -3490,7 +3496,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr" s="2">
+      <c r="H4" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B: Horror</t>
         </is>
@@ -3507,12 +3513,12 @@
           <t xml:space="preserve">blush</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="G5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Oh? A romance, then...</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr" s="2">
+      <c r="H5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -3529,12 +3535,12 @@
           <t xml:space="preserve">upset</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="2">
+      <c r="G6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I'm fine. Totally fine.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr" s="2">
+      <c r="H6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -3548,22 +3554,49 @@
       </c>
       <c r="F7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">The credits roll.</t>
+          <t xml:space="preserve">movie_night</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The two of you curl up as the movie starts.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Picture: shows only the CG, until "none"</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="D8" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The credits roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Template</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="2">
+      <c r="E9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">happy</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr" s="2">
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">That was fun. Back to writing?</t>
         </is>
@@ -3575,7 +3608,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -4065,10 +4098,22 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Picture</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reward art (CG). The scene shows only the picture, with the dialog on top, until another picture or "none".</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Choice</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr" s="2">
+      <c r="B46" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">On a You row, "A: button text" makes a choice. On later rows a letter (A) means "only if A was picked". Empty means everyone sees it, so paths rejoin.</t>
         </is>
@@ -6933,7 +6978,7 @@
   <sheetPr>
     <tabColor rgb="FFB08AD8"/>
   </sheetPr>
-  <dimension ref="A1:I166"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -6941,10 +6986,11 @@
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="80" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="80" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6975,20 +7021,25 @@
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Picture</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Line</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="1">
+      <c r="H1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Choice</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="1">
+      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Options</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
+      <c r="J1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -7005,12 +7056,12 @@
           <t xml:space="preserve">Whole goal 25%</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="2">
+      <c r="G2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Wow, you're already a quarter through. Good work. That's a substantial start, I'd say. Keep it up and you'll be done in no time. Shall we celebrate?</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr" s="2">
+      <c r="I2" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
         </is>
@@ -7022,14 +7073,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr" s="2">
+      <c r="G3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure! But... um... how?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="F4" t="inlineStr" s="2">
+      <c r="G4" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Hm... excellent question. How about we start by taking a break?</t>
         </is>
@@ -7041,7 +7092,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr" s="2">
+      <c r="G5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sounds good to me.</t>
         </is>
@@ -7053,14 +7104,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr" s="2">
+      <c r="G6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder turns on a game console and sits cross-legged in front of the couch. With a tilt of the analog stick, he sorts through a surprisingly large library of games...</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="F7" t="inlineStr" s="2">
+      <c r="G7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I have got to work on this backlog.</t>
         </is>
@@ -7072,14 +7123,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr" s="2">
+      <c r="G8" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">... he observes apologetically, sheepishly scratching his head before jolting to a stop on one.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="F9" t="inlineStr" s="2">
+      <c r="G9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Have you ever played a fighting game before?</t>
         </is>
@@ -7091,7 +7142,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr" s="2">
+      <c r="H10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A: No</t>
         </is>
@@ -7103,7 +7154,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr" s="2">
+      <c r="H11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B: Yes, and I'm good at them</t>
         </is>
@@ -7115,19 +7166,19 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr" s="2">
+      <c r="H12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C: Yes, but I'm not good at them</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="F13" t="inlineStr" s="2">
+      <c r="G13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ah, don't worry. This one is known for being beginner-friendly.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr" s="2">
+      <c r="H13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -7139,24 +7190,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr" s="2">
+      <c r="G14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Alright, I'll try it.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr" s="2">
+      <c r="H14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="F15" t="inlineStr" s="2">
+      <c r="G15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Oh, is that so? Then are you up for a challenge?</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr" s="2">
+      <c r="H15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7168,24 +7219,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr" s="2">
+      <c r="G16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr" s="2">
+      <c r="H16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="F17" t="inlineStr" s="2">
+      <c r="G17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ah, don't worry. I can teach you... if you'd like that, I mean.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr" s="2">
+      <c r="H17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -7197,19 +7248,19 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr" s="2">
+      <c r="G18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sounds good to me.</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr" s="2">
+      <c r="H18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="F19" t="inlineStr" s="2">
+      <c r="G19" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Then let's get started. I'll be him...</t>
         </is>
@@ -7221,26 +7272,26 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr" s="2">
+      <c r="G20" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder selects a scholarly-looking mage with a stoic expression.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="F21" t="inlineStr" s="2">
+      <c r="G21" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Who do you want to play?</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="F22" t="inlineStr" s="2">
+      <c r="G22" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Naples is an easy player for beginners to get a handle of. Would you like to try him?</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr" s="2">
+      <c r="H22" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
@@ -7252,12 +7303,12 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr" s="2">
+      <c r="G23" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure.</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr" s="2">
+      <c r="H23" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
@@ -7269,12 +7320,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr" s="2">
+      <c r="G24" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Slowly, I get used to the game.</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr" s="2">
+      <c r="H24" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
@@ -7286,24 +7337,24 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr" s="2">
+      <c r="G25" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder is kind, helpful, and gentle, going easy on me at first as he explains the very basics of movement, attacks, and strategy, but gradually taking off the kid gloves as I get used to the game.</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr" s="2">
+      <c r="H25" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="F26" t="inlineStr" s="2">
+      <c r="G26" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Wow, you've gotten so good already. I'm impressed.</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr" s="2">
+      <c r="H26" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
@@ -7315,36 +7366,36 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr" s="2">
+      <c r="G27" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Really? Thank you.</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr" s="2">
+      <c r="H27" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="F28" t="inlineStr" s="2">
+      <c r="G28" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Alright, one last thing to show you.</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr" s="2">
+      <c r="H28" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A, C</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="F29" t="inlineStr" s="2">
+      <c r="G29" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Zero December is good at ranged attacks, Lysandra is best for melee--</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr" s="2">
+      <c r="H29" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7356,12 +7407,12 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr" s="2">
+      <c r="G30" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I'll go with Castien.</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr" s="2">
+      <c r="H30" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7373,12 +7424,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr" s="2">
+      <c r="G31" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I pick up the nuances of the game quickly. Ryder turns out to be better than most people. Far better than I expected. What's more, he's also unexpectedly competitive.</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr" s="2">
+      <c r="H31" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7390,24 +7441,24 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr" s="2">
+      <c r="G32" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">We each take turns playfully trash-talking one another. As he nearly knocks my character out, offhandedly, he remarks,</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr" s="2">
+      <c r="H32" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="F33" t="inlineStr" s="2">
+      <c r="G33" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I seem to recall someone saying they were good at fighting games?</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr" s="2">
+      <c r="H33" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7419,24 +7470,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr" s="2">
+      <c r="G34" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Mind your own business.</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr" s="2">
+      <c r="H34" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="F35" t="inlineStr" s="2">
+      <c r="G35" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I don't know. I asked if you were up for a challenge and I'm actually beginning to feel quite cruel for it.</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr" s="2">
+      <c r="H35" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7448,12 +7499,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr" s="2">
+      <c r="G36" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">His special is almost completely powered up. I prepare to dodge the huge ball of energy as he activates it and...</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr" s="2">
+      <c r="H36" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7465,12 +7516,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr" s="2">
+      <c r="G37" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">it flies harmlessly up into the sky?</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr" s="2">
+      <c r="H37" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7482,24 +7533,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr" s="2">
+      <c r="G38" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Did you just... waste your special?</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr" s="2">
+      <c r="H38" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="F39" t="inlineStr" s="2">
+      <c r="G39" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I... that was on purpose. I was just testing you.</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr" s="2">
+      <c r="H39" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7511,12 +7562,12 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr" s="2">
+      <c r="G40" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Liar. So you were all talk!</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr" s="2">
+      <c r="H40" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7528,12 +7579,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr" s="2">
+      <c r="G41" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">And as I say that, I swoop in while he's vulnerable and finish him off.</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr" s="2">
+      <c r="H41" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -7545,7 +7596,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr" s="2">
+      <c r="G42" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">[PLACEHOLDER rest of the game-night scene, after "one last thing to show you"]</t>
         </is>
@@ -7563,12 +7614,12 @@
           <t xml:space="preserve">Whole goal 100%</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr" s="2">
+      <c r="G44" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">You did it. You're more determined than I imagined, honestly. Say... are you going to let me read it now?</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr" s="2">
+      <c r="I44" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
         </is>
@@ -7580,7 +7631,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr" s="2">
+      <c r="H45" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A: Absolutely not</t>
         </is>
@@ -7592,38 +7643,38 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr" s="2">
+      <c r="H46" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B: Sure</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="F47" t="inlineStr" s="2">
+      <c r="G47" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">It was worth asking. But seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr" s="2">
+      <c r="H47" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="F48" t="inlineStr" s="2">
+      <c r="G48" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Glad to hear. Seriously... I can't believe you did it... well, no, I always believed you could. Rather, I can't believe it happened so fast.</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr" s="2">
+      <c r="H48" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="F49" t="inlineStr" s="2">
+      <c r="G49" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I'm running out of ways to celebrate. Well, except one.</t>
         </is>
@@ -7635,14 +7686,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr" s="2">
+      <c r="G50" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">What is it?</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="F51" t="inlineStr" s="2">
+      <c r="G51" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Let's sit down first...</t>
         </is>
@@ -7654,14 +7705,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr" s="2">
+      <c r="G52" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">On the floor again, right?</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="F53" t="inlineStr" s="2">
+      <c r="G53" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">... No, on the couch.</t>
         </is>
@@ -7673,14 +7724,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr" s="2">
+      <c r="G54" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Really?!</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="F55" t="inlineStr" s="2">
+      <c r="G55" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes, is that strange...?</t>
         </is>
@@ -7692,21 +7743,21 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr" s="2">
+      <c r="G56" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Considering how weird you've been about it, yeah.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="F57" t="inlineStr" s="2">
+      <c r="G57" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ah, so you noticed my aversion to sitting on it... I suppose I wanted to keep it clean since it was the first thing I ever bought for myself...</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="F58" t="inlineStr" s="2">
+      <c r="G58" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">But, well, there's something more important than that now.</t>
         </is>
@@ -7718,14 +7769,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr" s="2">
+      <c r="G59" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Such as?</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="F60" t="inlineStr" s="2">
+      <c r="G60" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Well, about that... there's something I've been wanting to tell you, but I was worried about how you'd react...</t>
         </is>
@@ -7737,28 +7788,28 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr" s="2">
+      <c r="G61" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Go on.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="F62" t="inlineStr" s="2">
+      <c r="G62" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I just... I think I may have fallen for you.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="F63" t="inlineStr" s="2">
+      <c r="G63" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I feel so safe with you. And I want you to feel like that with me. I know I can be awkward, and talk too much, but... {player}, I love you. I want you to be mine, and I want to be yours. But...</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="F64" t="inlineStr" s="2">
+      <c r="G64" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I understand if you don't feel the same way--</t>
         </is>
@@ -7770,14 +7821,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr" s="2">
+      <c r="G65" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I close the distance between me and him and gently kiss him. His lips are soft and his body warm against mine.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="F66" t="inlineStr" s="2">
+      <c r="G66" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I wasn't expecting that. Do you...</t>
         </is>
@@ -7789,14 +7840,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr" s="2">
+      <c r="G67" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I do.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="F68" t="inlineStr" s="2">
+      <c r="G68" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">What?</t>
         </is>
@@ -7808,14 +7859,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr" s="2">
+      <c r="G69" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I love you, too.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="F70" t="inlineStr" s="2">
+      <c r="G70" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I...wasn't expecting that. Why?</t>
         </is>
@@ -7827,7 +7878,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr" s="2">
+      <c r="G71" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">The same reason you love me, dummy. You feel like home.</t>
         </is>
@@ -7839,7 +7890,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr" s="2">
+      <c r="G72" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I take his hands into mine.</t>
         </is>
@@ -7851,14 +7902,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr" s="2">
+      <c r="G73" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I want to be with you, too, Ryder. I'm just wondering.. what happened to the kuudere act you had at the beginning of the month?</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="F74" t="inlineStr" s="2">
+      <c r="G74" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Huh?</t>
         </is>
@@ -7870,7 +7921,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr" s="2">
+      <c r="G75" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Every few days you do this thing where you act like you're too cool for school.</t>
         </is>
@@ -7882,14 +7933,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr" s="2">
+      <c r="G76" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">"I suppose I can do my best to support you, but no promises made." "You're incredible. ...don't let it go to your head." And so on.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="F77" t="inlineStr" s="2">
+      <c r="G77" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Well... being an unabashed cheerleader isn't very cool, is it...?</t>
         </is>
@@ -7901,7 +7952,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr" s="2">
+      <c r="G78" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">[PLACEHOLDER rest of the confession scene]</t>
         </is>
@@ -7919,12 +7970,12 @@
           <t xml:space="preserve">Whole goal 50%</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr" s="2">
+      <c r="G80" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I wasn't sure you could do it, but here we are. Halfway through. You're incredible. ...don't let it go to your head. Now maybe we should take a break. Would you like to watch a movie?</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr" s="2">
+      <c r="I80" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
         </is>
@@ -7936,7 +7987,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr" s="2">
+      <c r="G81" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure!</t>
         </is>
@@ -7948,7 +7999,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr" s="2">
+      <c r="G82" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">As I leap towards the couch, Ryder grabs my arm and pulls me back, mid-air.</t>
         </is>
@@ -7960,14 +8011,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr" s="2">
+      <c r="G83" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Huh?</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="F84" t="inlineStr" s="2">
+      <c r="G84" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">We... uh, need popcorn.</t>
         </is>
@@ -7979,14 +8030,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr" s="2">
+      <c r="G85" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">... Right.</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="F86" t="inlineStr" s="2">
+      <c r="G86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Wait there.</t>
         </is>
@@ -7998,7 +8049,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr" s="2">
+      <c r="G87" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I wait approximately five minutes as Ryder finds and prepares popcorn for us. Finally he returns.</t>
         </is>
@@ -8010,14 +8061,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr" s="2">
+      <c r="G88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Can I sit now--</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="F89" t="inlineStr" s="2">
+      <c r="G89" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">No! I mean. Wouldn't it be more fun to sit on the ground?</t>
         </is>
@@ -8029,7 +8080,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr" s="2">
+      <c r="G90" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He demonstrates by sitting cross-legged on the ground and patting the space next to him. Confused, I sit down.</t>
         </is>
@@ -8041,14 +8092,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr" s="2">
+      <c r="G91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Okay then.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="F92" t="inlineStr" s="2">
+      <c r="G92" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Anyway. What type of movie would you like to watch?</t>
         </is>
@@ -8060,7 +8111,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr" s="2">
+      <c r="H93" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A: Romance</t>
         </is>
@@ -8072,7 +8123,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr" s="2">
+      <c r="H94" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B: Action</t>
         </is>
@@ -8084,19 +8135,19 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr" s="2">
+      <c r="H95" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C: Horror</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="F96" t="inlineStr" s="2">
+      <c r="G96" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Oh? If that's the case, then... well, there's one I've been meaning to watch...</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr" s="2">
+      <c r="H96" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8108,24 +8159,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr" s="2">
+      <c r="G97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">What's it called?</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr" s="2">
+      <c r="H97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="F98" t="inlineStr" s="2">
+      <c r="G98" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">The Notepad?</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr" s="2">
+      <c r="H98" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8137,24 +8188,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr" s="2">
+      <c r="G99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Oh, that's a classic.</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr" s="2">
+      <c r="H99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="F100" t="inlineStr" s="2">
+      <c r="G100" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">That's what I heard. So shall we?</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr" s="2">
+      <c r="H100" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8166,12 +8217,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr" s="2">
+      <c r="G101" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I nod and he starts the movie. He and I both intently watch a story about star-crossed lovers. As the credits roll, I'm sniffling. I look around and can't find Ryder.</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr" s="2">
+      <c r="H101" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8183,12 +8234,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr" s="2">
+      <c r="G102" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">But then there he is with a box of tissues, also looking teary eyed.</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr" s="2">
+      <c r="H102" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8200,24 +8251,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr" s="2">
+      <c r="G103" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Are you okay?</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr" s="2">
+      <c r="H103" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="F104" t="inlineStr" s="2">
+      <c r="G104" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I will be. Would you like a tissue?</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr" s="2">
+      <c r="H104" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
@@ -8229,36 +8280,36 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr" s="2">
+      <c r="G105" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure.</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr" s="2">
+      <c r="H105" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="F106" t="inlineStr" s="2">
+      <c r="G106" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Not the best movie we could've picked for a celebration but it certainly was an experience, wasn't it?</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr" s="2">
+      <c r="H106" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="F107" t="inlineStr" s="2">
+      <c r="G107" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I wonder if they have that movie I kept hearing about... They do!</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr" s="2">
+      <c r="H107" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8270,24 +8321,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr" s="2">
+      <c r="G108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Superguy?</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr" s="2">
+      <c r="H108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="F109" t="inlineStr" s="2">
+      <c r="G109" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes, it sounds fun, doesn't it? And the ratings are very good.</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr" s="2">
+      <c r="H109" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8299,12 +8350,12 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr" s="2">
+      <c r="G110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure, let's watch it then.</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr" s="2">
+      <c r="H110" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8316,12 +8367,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr" s="2">
+      <c r="G111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">As we watch the movie, sitting on the uncomfortable hardwood floor, Ryder's eyebrows contort further and further. Afterwards, he has a solid frown on his face.</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr" s="2">
+      <c r="H111" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8333,24 +8384,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr" s="2">
+      <c r="G112" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">You look like you have a lot of thoughts about the movie.</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr" s="2">
+      <c r="H112" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="F113" t="inlineStr" s="2">
+      <c r="G113" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I do.</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr" s="2">
+      <c r="H113" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8362,12 +8413,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr" s="2">
+      <c r="G114" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">What a cryptic response.</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr" s="2">
+      <c r="H114" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8379,36 +8430,36 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr" s="2">
+      <c r="G115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Such as...?</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr" s="2">
+      <c r="H115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="F116" t="inlineStr" s="2">
+      <c r="G116" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He's supposed to be a superhero but he's causing so much trouble! Just think about all the collateral damage he left!</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr" s="2">
+      <c r="H116" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="F117" t="inlineStr" s="2">
+      <c r="G117" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Even assuming nobody got hurt from when he threw the villain into that skyscraper, what about taxpayer money?!</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr" s="2">
+      <c r="H117" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
@@ -8420,36 +8471,36 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr" s="2">
+      <c r="G118" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">It's a movie. An explosive movie, but a movie.</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr" s="2">
+      <c r="H118" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="F119" t="inlineStr" s="2">
+      <c r="G119" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Fair enough. We won't always like the same things, I suppose.</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr" s="2">
+      <c r="H119" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="F120" t="inlineStr" s="2">
+      <c r="G120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure. I have no problem with that. None at all.</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr" s="2">
+      <c r="H120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8461,24 +8512,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr" s="2">
+      <c r="G121" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Then let's watch The Circle!</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr" s="2">
+      <c r="H121" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="F122" t="inlineStr" s="2">
+      <c r="G122" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Right.</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr" s="2">
+      <c r="H122" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8490,24 +8541,24 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr" s="2">
+      <c r="G123" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He says that but almost immediately as the movie starts...</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr" s="2">
+      <c r="H123" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="F124" t="inlineStr" s="2">
+      <c r="G124" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I think I should go make some popcorn.</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr" s="2">
+      <c r="H124" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8519,24 +8570,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr" s="2">
+      <c r="G125" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Nuh-uh, you're not getting out of this one.</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr" s="2">
+      <c r="H125" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="F126" t="inlineStr" s="2">
+      <c r="G126" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">But I--</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr" s="2">
+      <c r="H126" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8548,24 +8599,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr" s="2">
+      <c r="G127" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sit.</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr" s="2">
+      <c r="H127" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="F128" t="inlineStr" s="2">
+      <c r="G128" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I see...</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr" s="2">
+      <c r="H128" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8577,12 +8628,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr" s="2">
+      <c r="G129" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Even so, he averts his eyes the whole movie, tensing with every jumpscare... and looking terrified out of his mind. After the movie, he's skittish.</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr" s="2">
+      <c r="H129" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8594,12 +8645,12 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr" s="2">
+      <c r="G130" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">As he's reaching in the fridge for a bottle of water, I start talking and he jumps.</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr" s="2">
+      <c r="H130" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8611,24 +8662,24 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr" s="2">
+      <c r="G131" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder? You okay?</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr" s="2">
+      <c r="H131" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="F132" t="inlineStr" s="2">
+      <c r="G132" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes, I think I'll be okay. Let's just... I think I'm going to leave the light on tonight.</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr" s="2">
+      <c r="H132" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">C</t>
         </is>
@@ -8646,19 +8697,19 @@
           <t xml:space="preserve">Whole goal 75%</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr" s="2">
+      <c r="G134" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">You've got three quarters of your work done. That's the vast majority! I'm honestly impressed by your dedication.</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr" s="2">
+      <c r="I134" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">once</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="F135" t="inlineStr" s="2">
+      <c r="G135" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I think that deserves a treat. How about we go for frozen yogurt?</t>
         </is>
@@ -8670,7 +8721,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr" s="2">
+      <c r="G136" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sure!</t>
         </is>
@@ -8682,7 +8733,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr" s="2">
+      <c r="G137" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">When we arrive at the froyo place, Ryder holds the door open for me. We get tiny sample cups and push down the levers to dispense the froyo.</t>
         </is>
@@ -8694,7 +8745,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr" s="2">
+      <c r="G138" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">There are twelve different flavors and we spend time diligently sampling each and every one, trying to decide which one to put in our bowl. In the end, I decide on a flavor...</t>
         </is>
@@ -8706,7 +8757,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr" s="2">
+      <c r="G139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Then I see Ryder looking seriously pained, like he can't bear to part with any one flavor.</t>
         </is>
@@ -8718,14 +8769,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr" s="2">
+      <c r="G140" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Are you alright?</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="F141" t="inlineStr" s="2">
+      <c r="G141" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I'm fine. I'll just...</t>
         </is>
@@ -8737,14 +8788,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr" s="2">
+      <c r="G142" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He suddenly pulls a lever, releasing salted caramel froyo into his bowl.</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="F143" t="inlineStr" s="2">
+      <c r="G143" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Wait!</t>
         </is>
@@ -8756,14 +8807,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr" s="2">
+      <c r="G144" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He stops and adds cake batter flavor. And then cookies and cream. He sighs with relief.</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="F145" t="inlineStr" s="2">
+      <c r="G145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">That should be fine.</t>
         </is>
@@ -8775,7 +8826,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr" s="2">
+      <c r="G146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">When we're adding toppings, it's clear he's been struck by a similar indecision.</t>
         </is>
@@ -8787,7 +8838,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr" s="2">
+      <c r="G147" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">In the end, he piles on chocolate chips, corn flakes, caramel, marshmallow sauce, and cookie dough pieces, each neatly placed in their own section of the bowl.</t>
         </is>
@@ -8799,7 +8850,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr" s="2">
+      <c r="G148" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder pays for both of us.</t>
         </is>
@@ -8811,14 +8862,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr" s="2">
+      <c r="G149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Do you wanna go back home? We can sit on the couch, watch TV--</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="F150" t="inlineStr" s="2">
+      <c r="G150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">A-ah, I think I'd prefer to eat here. Outside.</t>
         </is>
@@ -8830,7 +8881,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr" s="2">
+      <c r="G151" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">No problem.</t>
         </is>
@@ -8842,7 +8893,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr" s="2">
+      <c r="G152" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Is it just me or did he get weird when I mentioned the couch?</t>
         </is>
@@ -8854,7 +8905,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr" s="2">
+      <c r="G153" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">We go outside and sit down. I dug into my frozen treat, only to eventually notice Ryder staring.</t>
         </is>
@@ -8866,14 +8917,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr" s="2">
+      <c r="G154" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Is there something on my face?</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="F155" t="inlineStr" s="2">
+      <c r="G155" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes. It's right there.</t>
         </is>
@@ -8885,7 +8936,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr" s="2">
+      <c r="G156" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He points at my face.</t>
         </is>
@@ -8897,14 +8948,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr" s="2">
+      <c r="G157" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Right here?</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="F158" t="inlineStr" s="2">
+      <c r="G158" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">No, there.</t>
         </is>
@@ -8916,14 +8967,14 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr" s="2">
+      <c r="G159" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Here?</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="F160" t="inlineStr" s="2">
+      <c r="G160" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ah, no, it's here...</t>
         </is>
@@ -8935,7 +8986,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr" s="2">
+      <c r="G161" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He reaches across the table and brushes his thumb gently near my mouth.</t>
         </is>
@@ -8947,14 +8998,14 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr" s="2">
+      <c r="G162" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">For some reason, I can feel my face heat up.</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="F163" t="inlineStr" s="2">
+      <c r="G163" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sorry, I shouldn't have done that.</t>
         </is>
@@ -8966,7 +9017,7 @@
           <t xml:space="preserve">You</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr" s="2">
+      <c r="G164" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">No, it's fine.</t>
         </is>
@@ -8978,7 +9029,7 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr" s="2">
+      <c r="G165" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">But the whole time, I can't forget the way it felt when he touched me.</t>
         </is>
@@ -8986,13 +9037,16 @@
     </row>
     <row r="166"/>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="D2:D500">
       <formula1>"Ryder,You,Narrator"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="E2:E500">
       <formula1>"blush,blushavert,flushed,glad,happy,muse,neutral,serious,shocked,smile,surprised,thinking,tired,upset,veryhappy"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="0" sqref="F2:F500">
+      <formula1>"none"</formula1>
+    </dataValidation>
   </dataValidations>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ryder: fill day 30 and day 31 lines, drop unused chocolate flag; scene docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/cutie-scripts.xlsx
+++ b/content/cutie-scripts.xlsx
@@ -5700,8 +5700,8 @@
       <c r="C28" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">{player}, do you like chocolate? If I woke up one day allergic to it, I don't know what I'd do...
-[A: Yeah!] Is that so? I do, too! Thanks for answering, anyway. I'll keep it in mind. [set likes chocolate = yes]
-[B: Not really] Really? I'll keep that in mind then... [set likes chocolate = no]</t>
+[A: Yeah!] Is that so? I do, too! Thanks for answering, anyway. I'll keep it in mind.
+[B: Not really] Really? I'll keep that in mind then...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="2">
@@ -5833,7 +5833,7 @@
         <is>
           <t xml:space="preserve">{blushavert} Morning. Er... do you remember anything I said to you last night?
 [A: You said something to me?] No, nothing of importance.
-[B: Yes, I do] [PLACEHOLDER Ryder reacts: player heard the confession]</t>
+[B: Yes, I do] {blushavert} You... heard that? Then I won't take it back. I meant every word.</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">{serious} [PLACEHOLDER last day of the month]</t>
+          <t xml:space="preserve">{serious} Last day, {player}. {words left} words to go. Whatever happens, I'm proud of you. Let's finish this together.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ryder: placeholder CGs in the four cutscenes; screenshot the CG part and gallery
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/cutie-scripts.xlsx
+++ b/content/cutie-scripts.xlsx
@@ -7104,6 +7104,11 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">game_night</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Ryder turns on a game console and sits cross-legged in front of the couch. With a tilt of the analog stick, he sorts through a surprisingly large library of games...</t>
@@ -7121,6 +7126,11 @@
       <c r="D8" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Narrator</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="2">
@@ -7821,6 +7831,11 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">the_couch</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">I close the distance between me and him and gently kiss him. His lips are soft and his body warm against mine.</t>
@@ -7838,6 +7853,11 @@
       <c r="D67" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">You</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
       <c r="G67" t="inlineStr" s="2">
@@ -8080,6 +8100,11 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">movie_night</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He demonstrates by sitting cross-legged on the ground and patting the space next to him. Confused, I sit down.</t>
@@ -8099,6 +8124,11 @@
       </c>
     </row>
     <row r="92">
+      <c r="F92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Anyway. What type of movie would you like to watch?</t>
@@ -8986,6 +9016,11 @@
           <t xml:space="preserve">Narrator</t>
         </is>
       </c>
+      <c r="F161" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">froyo_date</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">He reaches across the table and brushes his thumb gently near my mouth.</t>
@@ -9005,6 +9040,11 @@
       </c>
     </row>
     <row r="163">
+      <c r="F163" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
       <c r="G163" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Sorry, I shouldn't have done that.</t>

</xml_diff>

<commit_message>
Affection never drops when words are deleted; add words_deleted moments (100 and 1000 placeholders for Ryder)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/cutie-scripts.xlsx
+++ b/content/cutie-scripts.xlsx
@@ -4018,7 +4018,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Stage Friend   ·   Streak 7   ·   Idle 5 min   ·   Every 1000 words   ·   Random</t>
+          <t xml:space="preserve">Stage Friend   ·   Streak 7   ·   Idle 5 min   ·   Every 1000 words   ·   Deleted 100 words   ·   Random</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="2">
@@ -6803,7 +6803,7 @@
   <sheetPr>
     <tabColor rgb="FFB08AD8"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -6966,6 +6966,40 @@
       <c r="C10" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">{smile} Another thousand words. That makes {total words}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Deleted 100 words</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">{surprised} [PLACEHOLDER Ryder reacts: you deleted 100 words in one go]</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">wait 10 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Deleted 1000 words</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">{shocked} [PLACEHOLDER Ryder reacts: you deleted 1000 words in one go]</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">daily</t>
         </is>
       </c>
     </row>

</xml_diff>